<commit_message>
Gallery: photo details from the contact sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -505,7 +505,11 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Day 2025</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1630,7 +1634,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Itay's talk</t>
+          <t>Itay receives his MSc!</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1638,7 +1642,11 @@
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Itay</t>
@@ -1705,7 +1713,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Moving into our new office</t>
+          <t>Moving into our new office!</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Gallery: more photo details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -1293,7 +1293,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>Chemistry @ Sete</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1303,10 +1303,14 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Kasia</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1320,14 +1324,26 @@
           <t>20250715_135739.jpg</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Chemistry @ Sete</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Kasia, Renana</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
Gallery: photo details for 32 photos, remove 3 duplicates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo details" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Photo details'!$A$1:$G$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Photo details'!$A$1:$G$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0004.jpg</t>
+          <t>IMG-20250101-WA0007.jpg</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1456,7 +1456,11 @@
           <t>Croatia</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Shabu</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1467,75 +1471,95 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0006.jpg</t>
+          <t>WhatsApp Image 2026-09-10 at 9.47.53 AM.jpeg</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Talk at ICESAA3</t>
+          <t>CBOND</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Renana</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0007.jpg</t>
+          <t>WhatsApp Image 2026-09-11 at 2.16.39 PM.jpeg</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Talk at ICESAA3</t>
+          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Renana</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-10 at 9.47.53 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-11 at 1.47.55 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+        </is>
+      </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1546,7 +1570,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 2.16.39 PM.jpeg</t>
+          <t>WhatsApp Image 2026-09-11 at 2.30.10 PM.jpeg</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1566,7 +1590,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Ajeet, Renana</t>
+          <t>Ajeet</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
@@ -1579,12 +1603,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 1.47.55 PM.jpeg</t>
+          <t>WhatsApp Image 2026-09-06 at 5.37.56 PM (1).jpeg</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+          <t>Itay receives his MSc!</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1594,12 +1618,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>Technion</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Ajeet</t>
+          <t>Itay</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
@@ -1612,27 +1636,27 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 2.30.10 PM.jpeg</t>
+          <t>WhatsApp Image 2026-08-13 at 8.58.56 AM.jpeg</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+          <t>Amrita's Chem Sci is published!!</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>August 2026</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>Technion</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Ajeet</t>
+          <t>Renana, Amrita</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
@@ -1645,27 +1669,19 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-06 at 5.37.56 PM (1).jpeg</t>
+          <t>Eduardo Defense.jpg</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Itay receives his MSc!</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
+          <t>Eduardo's thesis defense</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Itay</t>
+          <t>Eduardo</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
@@ -1678,16 +1694,24 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-13 at 8.58.56 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr"/>
+          <t>20220615_124230.jpg</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Moving into our new office!</t>
+        </is>
+      </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
+          <t>June 2022</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1699,21 +1723,25 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Eduardo Defense.jpg</t>
+          <t>20220615_124701.jpg</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Eduardo's thesis defense</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo</t>
-        </is>
-      </c>
+          <t>Moving into our new office</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>June 2022</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1724,25 +1752,25 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>20220615_124230.jpg</t>
+          <t>20250323_102940.jpg</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Moving into our new office!</t>
+          <t>Fatimah's birthday</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>June 2022</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
+          <t>March 2025</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Fatimah</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1753,25 +1781,25 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>20220615_124701.jpg</t>
+          <t>20250323_103002.jpg</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Moving into our new office</t>
+          <t>Kasia's birthday</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>June 2022</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
+          <t>March 2025</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Kasia</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
@@ -1782,23 +1810,23 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>20250323_102940.jpg</t>
+          <t>20250714_132616.jpg</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Fatimah's birthday</t>
+          <t>Renana's birthday</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>July 2025</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Fatimah</t>
+          <t>Renana</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -1811,23 +1839,23 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>20250323_103002.jpg</t>
+          <t>IMG-20250101-WA0025.jpg</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Kasia's birthday</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>March 2025</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Kasia</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
@@ -1840,25 +1868,21 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>20250714_132616.jpg</t>
+          <t>IMG-20250101-WA0026.jpg</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Renana's birthday</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Renana</t>
-        </is>
-      </c>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -1869,12 +1893,20 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0025.jpg</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr"/>
+          <t>IMG-20250101-WA0027.jpg</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
       <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr"/>
     </row>
@@ -1886,11 +1918,15 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0026.jpg</t>
+          <t>WhatsApp Image 2026-08-30 at 10.52.54 AM.jpeg</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>August 2026</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr"/>
@@ -1903,11 +1939,15 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0027.jpg</t>
+          <t>WhatsApp Image 2026-08-30 at 10.53.10 AM.jpeg</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>August 2026</t>
+        </is>
+      </c>
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr"/>
@@ -1915,35 +1955,55 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0028.jpg</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
+          <t>20220915_230425.jpg</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Getting to see Greta in Cambridge!</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>September 2022</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Cambridge, UK</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Greta, Renana</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-30 at 10.52.54 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr"/>
+          <t>20250714_155815.jpg</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Renana's Birthday (we won't say how old)</t>
+        </is>
+      </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>July 2025</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -1953,22 +2013,30 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-30 at 10.53.10 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr"/>
+          <t>20250822_210225.jpg</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Catching up with Alex!</t>
+        </is>
+      </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>August 2025</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Alex W., Renana</t>
+        </is>
+      </c>
       <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -1979,17 +2047,25 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>20220915_230425.jpg</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr"/>
+          <t>PXL_20250904_111646408.PORTRAIT.jpg</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Kasia's Birthday :-)</t>
+        </is>
+      </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>September 2022</t>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Kasia</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2000,17 +2076,29 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>20250714_155815.jpg</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr"/>
+          <t>PXL_20250911_190210657.jpg</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>With Sasha at ESOR2025</t>
+        </is>
+      </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Padova</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Tsybizova, Renana</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
@@ -2021,17 +2109,25 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>20250822_210225.jpg</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr"/>
+          <t>PXL_20251010_111046551.jpg</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>August 2025</t>
+          <t>October 2025</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Itay</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2042,17 +2138,25 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250904_111646408.PORTRAIT.jpg</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr"/>
+          <t>PXL_20251010_111056036.jpg</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
+          <t>October 2025</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Shabu</t>
+        </is>
+      </c>
       <c r="G60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
@@ -2063,13 +2167,13 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250911_190210657.jpg</t>
+          <t>PXL_20260129_090902476.jpg</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
+          <t>January 2026</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr"/>
@@ -2084,17 +2188,25 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251010_111046551.jpg</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2025-10-10 at 12.59.25 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
           <t>October 2025</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Ajeet, Shabu, Itay</t>
+        </is>
+      </c>
       <c r="G62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
@@ -2105,16 +2217,24 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251010_111056036.jpg</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM2.jpeg</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>CBOND 2026 gala night</t>
+        </is>
+      </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>October 2025</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr"/>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
     </row>
@@ -2126,13 +2246,17 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>PXL_20260129_090902476.jpg</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.53.29 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>January 2026</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
@@ -2147,13 +2271,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2025-10-10 at 12.59.25 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.29 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>October 2025</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr"/>
@@ -2168,20 +2296,20 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM2.jpeg</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.42 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Brussels, Belgium</t>
-        </is>
-      </c>
+      <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
     </row>
@@ -2193,10 +2321,14 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.53.29 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.52 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2214,10 +2346,14 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.29 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.55 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2235,10 +2371,14 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.42 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2256,10 +2396,14 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.52 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM2.jpeg</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2272,60 +2416,80 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>with_our_friends</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.55 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr"/>
+          <t>Anya_WATOC_2022.jpg</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>WATOC 2022</t>
+        </is>
+      </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr"/>
-      <c r="F71" s="2" t="inlineStr"/>
+          <t>July 2022</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Anya</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>with_our_friends</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr"/>
+          <t>20220702_120019.jpg</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>WATOC 2022</t>
+        </is>
+      </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr"/>
+          <t>July 2022</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>with_our_friends</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM2.jpeg</t>
+          <t>20250709_170226.jpg</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>July 2025</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr"/>
@@ -2340,29 +2504,17 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Anya_WATOC_2022.jpg</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>WATOC 2022</t>
-        </is>
-      </c>
+          <t>20250710_093403.jpg</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>July 2022</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, Canada</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Anya</t>
-        </is>
-      </c>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
@@ -2373,24 +2525,16 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>20220702_120019.jpg</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>WATOC 2022</t>
-        </is>
-      </c>
+          <t>20250710_200322.jpg</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>July 2022</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, Canada</t>
-        </is>
-      </c>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr"/>
     </row>
@@ -2402,13 +2546,13 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>20250709_170226.jpg</t>
+          <t>PXL_20250910_063029882.MP.jpg</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
@@ -2423,13 +2567,13 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>20250710_093403.jpg</t>
+          <t>PXL_20251013_175543692.MP.jpg</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
+          <t>October 2025</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
@@ -2444,13 +2588,13 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>20250710_200322.jpg</t>
+          <t>PXL_20251210_075901835.jpg</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
+          <t>December 2025</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
@@ -2465,88 +2609,25 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250910_063029882.MP.jpg</t>
+          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM.jpeg</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr"/>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr"/>
     </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>with_our_friends</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>PXL_20251013_175543692.MP.jpg</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr"/>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>October 2025</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>with_our_friends</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>PXL_20251210_075901835.jpg</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr"/>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>December 2025</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr"/>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>with_our_friends</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr"/>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>Brussels, Belgium</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G82"/>
+  <autoFilter ref="A1:G79"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2626,9 +2707,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId81"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Gallery: details for With Our Friends
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -2441,7 +2441,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Renana, Anya</t>
+          <t>Renana, Anya Grynova</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
@@ -2472,7 +2472,11 @@
           <t>Vancouver, Canada</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>ORCA</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2486,14 +2490,26 @@
           <t>20250709_170226.jpg</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr"/>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
           <t>July 2025</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr"/>
-      <c r="F73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Peter Schreiner</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
@@ -2507,14 +2523,26 @@
           <t>20250710_093403.jpg</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
           <t>July 2025</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Peter Chen, Peter Schreiner</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
@@ -2528,14 +2556,26 @@
           <t>20250710_200322.jpg</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
           <t>July 2025</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr"/>
-      <c r="F75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Tsybizova, Renana</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
@@ -2549,14 +2589,26 @@
           <t>PXL_20250910_063029882.MP.jpg</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>ESOR 2025</t>
+        </is>
+      </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
           <t>September 2025</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Padova</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Amnon Stanger, Roy Shenhar</t>
+        </is>
+      </c>
       <c r="G76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
@@ -2570,14 +2622,26 @@
           <t>PXL_20251013_175543692.MP.jpg</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr"/>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Liebig Lectureship Tour</t>
+        </is>
+      </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
           <t>October 2025</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Babis Pappas, Daniel Werz</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
@@ -2591,14 +2655,26 @@
           <t>PXL_20251210_075901835.jpg</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Solvay Workshop</t>
+        </is>
+      </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
           <t>December 2025</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Irena Stara, Judy Wu, Renana</t>
+        </is>
+      </c>
       <c r="G78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
@@ -2612,7 +2688,11 @@
           <t>WhatsApp Image 2026-09-10 at 9.46.57 AM.jpeg</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr"/>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>CBOND 2026</t>
+        </is>
+      </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2623,7 +2703,11 @@
           <t>Brussels, Belgium</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Ephrath Solel, Renana, Ajeet</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gallery: 21 new photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo details" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Photo details'!$A$1:$G$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Photo details'!$A$1:$G$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -762,269 +762,173 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ICS_1_2026.jpg</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>ICS Annual Meeting</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>February 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Tel Aviv, Israel</t>
-        </is>
-      </c>
+          <t>BVDZ1484.JPG</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>ICS_2_2026.jpg</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>ICS Annual Meeting</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>February 2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Tel Aviv, Israel</t>
-        </is>
-      </c>
+          <t>IFBT2444.JPG</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>ICS_3_2026.jpg</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>ICS Annual Meeting</t>
-        </is>
-      </c>
+          <t>IMG_0401.HEIC</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>February 2026</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Tel Aviv, Israel</t>
-        </is>
-      </c>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>ICS_4_2026.jpg</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>ICS Annual Meeting</t>
-        </is>
-      </c>
+          <t>IMG_0407.HEIC</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>February 2026</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Tel Aviv, Israel</t>
-        </is>
-      </c>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>ICS_5_2026.jpg</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>ICS Annual Meeting</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>February 2026</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Tel Aviv, Israel</t>
-        </is>
-      </c>
+          <t>MCCN1945.JPG</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>fatimah poster.jpg</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>ICESAA3 conference</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>July 2024</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Fatimah</t>
-        </is>
-      </c>
+          <t>NYCE6410.JPG</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0012.jpg</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>ICESAA3 conference</t>
-        </is>
-      </c>
+          <t>Nitz.Z-927316.jpg</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Fatimah</t>
-        </is>
-      </c>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0005.jpg</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>ICESAA3 conference</t>
-        </is>
-      </c>
+          <t>Nitz.Z-927322.jpg</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>we_love_our_science</t>
+          <t>through_the_years</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0008.jpg</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>ICESAA3 conference</t>
-        </is>
-      </c>
+          <t>Nitz.Z-9309745.jpg</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1036,22 +940,22 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0010.jpg</t>
+          <t>ICS_1_2026.jpg</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ICESAA3 conference</t>
+          <t>ICS Annual Meeting</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>February 2026</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Tel Aviv, Israel</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1065,21 +969,25 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>fatimah poster2.jpg</t>
+          <t>ICS_2_2026.jpg</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Poster presentation</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Fatimah</t>
-        </is>
-      </c>
+          <t>ICS Annual Meeting</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>February 2026</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Tel Aviv, Israel</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1090,29 +998,25 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Eduardo poster.jpg</t>
+          <t>ICS_4_2026.jpg</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICS Annual Meeting</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>February 2026</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo</t>
-        </is>
-      </c>
+          <t>Tel Aviv, Israel</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1123,29 +1027,25 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Itay poster.jpg</t>
+          <t>ICS_5_2026.jpg</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICS Annual Meeting</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>February 2026</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Itay</t>
-        </is>
-      </c>
+          <t>Tel Aviv, Israel</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1156,27 +1056,27 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Shabu and Itay poster.jpg</t>
+          <t>fatimah poster.jpg</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICESAA3 conference</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Shabu, Itay</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1189,27 +1089,27 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Shabu poster.jpg</t>
+          <t>IMG-20250101-WA0012.jpg</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICESAA3 conference</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Shabu</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1222,29 +1122,25 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Shany Poster.jpg</t>
+          <t>IMG-20250101-WA0005.jpg</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICESAA3 conference</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Shany</t>
-        </is>
-      </c>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1255,29 +1151,25 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Shany poster2.jpg</t>
+          <t>IMG-20250101-WA0008.jpg</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Faculty Day</t>
+          <t>ICESAA3 conference</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Schulich Faculty of Chemistry, Technion</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Shany</t>
-        </is>
-      </c>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1288,29 +1180,25 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0013.jpg</t>
+          <t>IMG-20250101-WA0010.jpg</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Chemistry @ Sete</t>
+          <t>ICESAA3 conference</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Kasia</t>
-        </is>
-      </c>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1321,27 +1209,19 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>20250715_135739.jpg</t>
+          <t>fatimah poster2.jpg</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Chemistry @ Sete</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
+          <t>Poster presentation</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Kasia, Renana</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
@@ -1354,17 +1234,29 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>20250715_135812.jpg</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+          <t>Eduardo poster.jpg</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Day</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Schulich Faculty of Chemistry, Technion</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Eduardo</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1375,17 +1267,29 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>20250715_135833.jpg</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
+          <t>Itay poster.jpg</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Day</t>
+        </is>
+      </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Schulich Faculty of Chemistry, Technion</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Itay</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1396,17 +1300,29 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>20250715_140001.jpg</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
+          <t>Shabu and Itay poster.jpg</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Day</t>
+        </is>
+      </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Schulich Faculty of Chemistry, Technion</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Itay</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1417,17 +1333,29 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>20250715_140013.jpg</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
+          <t>Shabu poster.jpg</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Day</t>
+        </is>
+      </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Schulich Faculty of Chemistry, Technion</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Shabu</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1438,27 +1366,27 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0007.jpg</t>
+          <t>Shany Poster.jpg</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Talk at ICESAA3</t>
+          <t>Faculty Day</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Schulich Faculty of Chemistry, Technion</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Shabu</t>
+          <t>Shany</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -1471,27 +1399,27 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-10 at 9.47.53 AM.jpeg</t>
+          <t>Shany poster2.jpg</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>CBOND</t>
+          <t>Faculty Day</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Brussels</t>
+          <t>Schulich Faculty of Chemistry, Technion</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Ajeet, Renana</t>
+          <t>Shany</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
@@ -1499,32 +1427,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 2.16.39 PM.jpeg</t>
+          <t>IMG-20250101-WA0013.jpg</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+          <t>Chemistry @ Sete</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Ajeet, Renana</t>
+          <t>Kasia</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -1532,32 +1460,32 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 1.47.55 PM.jpeg</t>
+          <t>20250715_135739.jpg</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+          <t>Chemistry @ Sete</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Brussels, Belgium</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Ajeet</t>
+          <t>Kasia, Renana</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
@@ -1565,268 +1493,212 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-11 at 2.30.10 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
-        </is>
-      </c>
+          <t>20250715_135812.jpg</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Brussels, Belgium</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Ajeet</t>
-        </is>
-      </c>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-06 at 5.37.56 PM (1).jpeg</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Itay receives his MSc!</t>
-        </is>
-      </c>
+          <t>20250715_135833.jpg</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Itay</t>
-        </is>
-      </c>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-13 at 8.58.56 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Amrita's Chem Sci is published!!</t>
-        </is>
-      </c>
+          <t>20250715_140001.jpg</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Amrita</t>
-        </is>
-      </c>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Eduardo Defense.jpg</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo's thesis defense</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>20250715_140013.jpg</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo</t>
-        </is>
-      </c>
+      <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>20220615_124230.jpg</t>
+          <t>IMG-20250101-WA0007.jpg</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Moving into our new office!</t>
+          <t>Talk at ICESAA3</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>June 2022</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr"/>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Shabu</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>20220615_124701.jpg</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Moving into our new office</t>
-        </is>
-      </c>
+          <t>Nitz.Z-927515.jpg</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>June 2022</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Technion</t>
-        </is>
-      </c>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>20250323_102940.jpg</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Fatimah's birthday</t>
-        </is>
-      </c>
+          <t>Nitz.Z-9309734.jpg</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>June 2026</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Fatimah</t>
-        </is>
-      </c>
+      <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>20250323_103002.jpg</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Kasia's birthday</t>
-        </is>
-      </c>
+          <t>Nitz.Z-9309740.jpg</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>June 2026</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Kasia</t>
-        </is>
-      </c>
+      <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>our_milestones</t>
+          <t>we_love_our_science</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>20250714_132616.jpg</t>
+          <t>WhatsApp Image 2026-09-10 at 9.47.53 AM.jpeg</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Renana's birthday</t>
+          <t>CBOND</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr"/>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Renana</t>
+          <t>Ajeet, Renana</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -1839,23 +1711,27 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0025.jpg</t>
+          <t>WhatsApp Image 2026-09-11 at 2.16.39 PM.jpeg</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Fatimah's MSc Seminar</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
+          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Technion</t>
+          <t>Brussels, Belgium</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Fatimah</t>
+          <t>Ajeet, Renana</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
@@ -1868,21 +1744,29 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0026.jpg</t>
+          <t>WhatsApp Image 2026-09-11 at 1.47.55 PM.jpeg</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Fatimah's MSc Seminar</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr"/>
+          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet</t>
+        </is>
+      </c>
       <c r="G50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -1893,21 +1777,29 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>IMG-20250101-WA0027.jpg</t>
+          <t>WhatsApp Image 2026-09-11 at 2.30.10 PM.jpeg</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Fatimah's MSc Seminar</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr"/>
+          <t>Chemistry Poster Prize for Ajeet at CBOND 2026</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Technion</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet</t>
+        </is>
+      </c>
       <c r="G51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
@@ -1918,17 +1810,29 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-30 at 10.52.54 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-09-06 at 5.37.56 PM (1).jpeg</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Itay receives his MSc!</t>
+        </is>
+      </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Itay</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -1939,48 +1843,52 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-08-30 at 10.53.10 AM.jpeg</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr"/>
+          <t>WhatsApp Image 2026-08-13 at 8.58.56 AM.jpeg</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Amrita's Chem Sci is published!!</t>
+        </is>
+      </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Amrita</t>
+        </is>
+      </c>
       <c r="G53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>20220915_230425.jpg</t>
+          <t>Eduardo Defense.jpg</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Getting to see Greta in Cambridge!</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>September 2022</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Cambridge, UK</t>
-        </is>
-      </c>
+          <t>Eduardo's thesis defense</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Greta, Renana</t>
+          <t>Eduardo</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
@@ -1988,82 +1896,86 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>20250714_155815.jpg</t>
+          <t>20220615_124230.jpg</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Renana's Birthday (we won't say how old)</t>
+          <t>Moving into our new office!</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr"/>
+          <t>June 2022</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>20250822_210225.jpg</t>
+          <t>20220615_124701.jpg</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Catching up with Alex!</t>
+          <t>Moving into our new office</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>August 2025</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>Alex W., Renana</t>
-        </is>
-      </c>
+          <t>June 2022</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250904_111646408.PORTRAIT.jpg</t>
+          <t>20250323_102940.jpg</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Kasia's Birthday :-)</t>
+          <t>Fatimah's birthday</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
+          <t>March 2025</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Kasia</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr"/>
@@ -2071,32 +1983,28 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250911_190210657.jpg</t>
+          <t>20250323_103002.jpg</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>With Sasha at ESOR2025</t>
+          <t>Kasia's birthday</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Padova</t>
-        </is>
-      </c>
+          <t>March 2025</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Tsybizova, Renana</t>
+          <t>Kasia</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
@@ -2104,28 +2012,28 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251010_111046551.jpg</t>
+          <t>20250714_132616.jpg</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Keren's Wedding!</t>
+          <t>Renana's birthday</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>October 2025</t>
+          <t>July 2025</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Ajeet, Itay</t>
+          <t>Renana</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
@@ -2133,28 +2041,28 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251010_111056036.jpg</t>
+          <t>IMG-20250101-WA0025.jpg</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Keren's Wedding!</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>October 2025</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Renana, Shabu</t>
+          <t>Fatimah</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
@@ -2162,98 +2070,86 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>PXL_20260129_090902476.jpg</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>January 2026</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr"/>
+          <t>IMG-20250101-WA0026.jpg</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2025-10-10 at 12.59.25 PM.jpeg</t>
+          <t>IMG-20250101-WA0027.jpg</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Keren's Wedding!</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>October 2025</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Ajeet, Shabu, Itay</t>
-        </is>
-      </c>
+          <t>Fatimah's MSc Seminar</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM2.jpeg</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>CBOND 2026 gala night</t>
-        </is>
-      </c>
+          <t>IMG_0252.HEIC</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Brussels, Belgium</t>
-        </is>
-      </c>
+      <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.53.29 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Paint by Numbers Night!!</t>
-        </is>
-      </c>
+          <t>IMG_0386.HEIC</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2266,19 +2162,15 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.29 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Paint by Numbers Night!!</t>
-        </is>
-      </c>
+          <t>IMG_0396.HEIC</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
@@ -2291,24 +2183,16 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.42 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Paint by Numbers Night!!</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>September 2026</t>
-        </is>
-      </c>
+          <t>Renana_birthday.png</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
@@ -2316,22 +2200,18 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.52 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Paint by Numbers Night!!</t>
-        </is>
-      </c>
+          <t>WhatsApp Image 2026-08-30 at 10.52.54 AM.jpeg</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>August 2026</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr"/>
@@ -2341,22 +2221,18 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>having_a_blast</t>
+          <t>our_milestones</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.55 PM.jpeg</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Paint by Numbers Night!!</t>
-        </is>
-      </c>
+          <t>WhatsApp Image 2026-08-30 at 10.53.10 AM.jpeg</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>August 2026</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr"/>
@@ -2371,21 +2247,29 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM.jpeg</t>
+          <t>20220915_230425.jpg</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Paint by Numbers Night!!</t>
+          <t>Getting to see Greta in Cambridge!</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="inlineStr"/>
+          <t>September 2022</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Cambridge, UK</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Greta, Renana</t>
+        </is>
+      </c>
       <c r="G69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
@@ -2396,17 +2280,17 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM2.jpeg</t>
+          <t>20250714_155815.jpg</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Paint by Numbers Night!!</t>
+          <t>Renana's Birthday (we won't say how old)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>July 2025</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr"/>
@@ -2416,32 +2300,28 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Anya_WATOC_2022.jpg</t>
+          <t>20250822_210225.jpg</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>WATOC 2022</t>
+          <t>Catching up with Alex!</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>July 2022</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, Canada</t>
-        </is>
-      </c>
+          <t>August 2025</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Renana, Anya Grynova</t>
+          <t>Alex W., Renana</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
@@ -2449,197 +2329,133 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>20220702_120019.jpg</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>WATOC 2022</t>
-        </is>
-      </c>
+          <t>IMG20260502111949.jpg</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>July 2022</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, Canada</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>ORCA</t>
-        </is>
-      </c>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>20250709_170226.jpg</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Peter Chen Symposium</t>
-        </is>
-      </c>
+          <t>IMG20260502111952.jpg</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>ETH Zurich</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Peter Schreiner</t>
-        </is>
-      </c>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>20250710_093403.jpg</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Peter Chen Symposium</t>
-        </is>
-      </c>
+          <t>IMG20260703105516.jpg</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>ETH Zurich</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Peter Chen, Peter Schreiner</t>
-        </is>
-      </c>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>20250710_200322.jpg</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Peter Chen Symposium</t>
-        </is>
-      </c>
+          <t>IMG_0420.HEIC</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>July 2025</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Zurich</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>Alexandra Tsybizova, Renana</t>
-        </is>
-      </c>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>PXL_20250910_063029882.MP.jpg</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>ESOR 2025</t>
-        </is>
-      </c>
+          <t>IMG_0429.HEIC</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>September 2025</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>Padova</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>Renana, Amnon Stanger, Roy Shenhar</t>
-        </is>
-      </c>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251013_175543692.MP.jpg</t>
+          <t>PXL_20250904_111646408.PORTRAIT.jpg</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Liebig Lectureship Tour</t>
+          <t>Kasia's Birthday :-)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>October 2025</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Freiburg</t>
-        </is>
-      </c>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Renana, Babis Pappas, Daniel Werz</t>
+          <t>Kasia</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr"/>
@@ -2647,32 +2463,32 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>with_our_friends</t>
+          <t>having_a_blast</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>PXL_20251210_075901835.jpg</t>
+          <t>PXL_20250911_190210657.jpg</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Solvay Workshop</t>
+          <t>With Sasha at ESOR2025</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>December 2025</t>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Brussels</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Irena Stara, Judy Wu, Renana</t>
+          <t>Alexandra Tsybizova, Renana</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
@@ -2680,38 +2496,614 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20251010_111046551.jpg</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Itay</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20251010_111056036.jpg</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Shabu</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20260129_090902476.jpg</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>January 2026</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2025-10-10 at 12.59.25 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Keren's Wedding!</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Ajeet, Shabu, Itay</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-10 at 9.46.57 AM2.jpeg</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>CBOND 2026 gala night</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, Belgium</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.53.29 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.29 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.42 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.52 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.55 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM.jpeg</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>having_a_blast</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Image 2026-09-16 at 8.59.56 PM2.jpeg</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Paint by Numbers Night!!</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
           <t>with_our_friends</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Anya_WATOC_2022.jpg</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>WATOC 2022</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>July 2022</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Anya Grynova</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>20220702_120019.jpg</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>WATOC 2022</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>July 2022</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>ORCA</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>20250709_170226.jpg</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Peter Schreiner</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>20250710_093403.jpg</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Peter Chen, Peter Schreiner</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>20250710_200322.jpg</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Peter Chen Symposium</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Tsybizova, Renana</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20250910_063029882.MP.jpg</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>ESOR 2025</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Padova</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Amnon Stanger, Roy Shenhar</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20251013_175543692.MP.jpg</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Liebig Lectureship Tour</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Babis Pappas, Daniel Werz</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>PXL_20251210_075901835.jpg</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Solvay Workshop</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Irena Stara, Judy Wu, Renana</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>with_our_friends</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>WhatsApp Image 2026-09-10 at 9.46.57 AM.jpeg</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>CBOND 2026</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>Brussels, Belgium</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>Ephrath Solel, Renana, Ajeet</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G79"/>
+  <autoFilter ref="A1:G99"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2791,6 +3183,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Gallery: details for 4 photos from the group dashboard
Faculty Research Day 2026 (2 photos) and Shabu's farewell (2 photos):
event, place and people, suggested by group members and approved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -804,14 +804,26 @@
           <t>IMG_0401.HEIC</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Shabu's Farewell Lunch</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Japanika, Haifa</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Pallavi, Elad, Shabu, Renana, Amrita, Fatimah, Ruth, Keren, Itay</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
@@ -825,14 +837,26 @@
           <t>IMG_0407.HEIC</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Shabu's last day at Poranne Group</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Poranne Group Office, Technion</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Renana, Shabu, Amrita, Pallavi</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -880,14 +904,26 @@
           <t>Nitz.Z-927316.jpg</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Elad, Fatimah, Renana, Amrita, Pallavi, Ajeet</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -901,14 +937,26 @@
           <t>Nitz.Z-927322.jpg</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Elad, Fatimah, Renana, Amrita, Pallavi, Ajeet</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Gallery details for 20 photos; profile panels on the People page
- Gallery: event, place and people for 20 photos, approved in the dashboard
- People: cards and hexagons with data-profile open a panel with bio,
  research interests, email (if the person chose to show it) and links;
  first profiles for Amrita and Ajeet
- apply_dashboard_export.py publishes approved profiles to
  tools/people_profiles.json / assets/js/people-profiles-data.js, and no
  longer fails on a second export from the same day

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/photo_gallery/photo_details.xlsx
+++ b/photo_gallery/photo_details.xlsx
@@ -970,14 +970,26 @@
           <t>Nitz.Z-9309745.jpg</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Elad, Fatimah, Renana, Amrita, Pallavi, Ajeet</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1666,14 +1678,26 @@
           <t>Nitz.Z-927515.jpg</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Brain storming session, Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Pallavi, Ajeet</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
@@ -1687,14 +1711,26 @@
           <t>Nitz.Z-9309734.jpg</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Poster Presentation, Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Renana</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
@@ -1708,14 +1744,26 @@
           <t>Nitz.Z-9309740.jpg</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Research Day 2026</t>
+        </is>
+      </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Renana, Ajeet</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2197,14 +2245,26 @@
           <t>IMG_0386.HEIC</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Shabu receiving his farewell gift :)</t>
+        </is>
+      </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Fatimah</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
@@ -2218,14 +2278,26 @@
           <t>IMG_0396.HEIC</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Shabu with his Project students</t>
+        </is>
+      </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Keren, Shabu, Ruth</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
@@ -2239,10 +2311,26 @@
           <t>Renana_birthday.png</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Our beloved Renana's birthday blast :)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Fatimah, Pallavi, Amrita, Renana, Ajeet, Shabu, Ruth</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
@@ -2256,14 +2344,26 @@
           <t>WhatsApp Image 2026-08-30 at 10.52.54 AM.jpeg</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr"/>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Amrita's Birthday</t>
+        </is>
+      </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr"/>
-      <c r="F67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Pallavi, Shabu, Renana, Amrita, Ajeet</t>
+        </is>
+      </c>
       <c r="G67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
@@ -2277,14 +2377,26 @@
           <t>WhatsApp Image 2026-08-30 at 10.53.10 AM.jpeg</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr"/>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Amrita's Birthday</t>
+        </is>
+      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Pallavi, Shabu, Renana, Amrita, Ajeet</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
@@ -2385,14 +2497,26 @@
           <t>IMG20260502111949.jpg</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Exploring the desert</t>
+        </is>
+      </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Negev, Israel</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Amrita, Ajeet</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2406,14 +2530,26 @@
           <t>IMG20260502111952.jpg</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr"/>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Beyond the lab, exploring Israel</t>
+        </is>
+      </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr"/>
-      <c r="F73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Negev, Israel</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Amrita, Ajeet</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
@@ -2427,14 +2563,26 @@
           <t>IMG20260703105516.jpg</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Summer trip!</t>
+        </is>
+      </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Beit She'an, Israel</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Ajeet</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
@@ -2448,14 +2596,26 @@
           <t>IMG_0420.HEIC</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Bowling Session: Shabu showing his magical trick!!!</t>
+        </is>
+      </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr"/>
-      <c r="F75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Shabu</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
@@ -2469,14 +2629,26 @@
           <t>IMG_0429.HEIC</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Group activity: Bowling night!!!</t>
+        </is>
+      </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Amrita, Renana, Ron, Yoni, Shabu</t>
+        </is>
+      </c>
       <c r="G76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
@@ -2610,14 +2782,26 @@
           <t>PXL_20260129_090902476.jpg</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr"/>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Shabu's birthday :)</t>
+        </is>
+      </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
           <t>January 2026</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr"/>
-      <c r="F81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Amrita, Ajeet, Shabu, Pallavi, Renana</t>
+        </is>
+      </c>
       <c r="G81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
@@ -2675,7 +2859,11 @@
           <t>Brussels, Belgium</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Renana, Ajeet</t>
+        </is>
+      </c>
       <c r="G83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
@@ -2724,8 +2912,16 @@
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr"/>
-      <c r="F85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Ajeet, Shabu, Renana, Fatimah, Amrita, Pallavi</t>
+        </is>
+      </c>
       <c r="G85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
@@ -2799,8 +2995,16 @@
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr"/>
-      <c r="F88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Shabu, Fatimah, Renana, Amrita, Pallavi, Ajeet</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
@@ -2824,8 +3028,16 @@
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr"/>
-      <c r="F89" s="2" t="inlineStr"/>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Pallavi, Shabu, Renana, Amrita, Ajeet, Fatimah</t>
+        </is>
+      </c>
       <c r="G89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
@@ -2849,8 +3061,16 @@
           <t>September 2026</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr"/>
-      <c r="F90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Technion</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Pallavi, Shabu, Renana, Amrita, Ajeet, Fatimah</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="inlineStr"/>
     </row>
     <row r="91">

</xml_diff>